<commit_message>
Fixed problem with original spreadsheet.
Changed:
  Sheet SNCImport cell C6
  Sheet Analysis cells H15 through 20 and I15 through 20
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\tmp\aqaExcel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80931850-81B2-401E-9994-56459919E5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DCC3515-EBC0-4E82-919B-E1954EDF74D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-315" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -1000,6 +1000,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1017,17 +1028,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3298,17 +3298,17 @@
         <f>Analysis!V5+Analysis!V$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E5" s="50" t="s">
+      <c r="E5" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-      <c r="L5" s="49"/>
-      <c r="M5" s="49"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="33" t="s">
@@ -3318,15 +3318,15 @@
         <f>Analysis!X5+Analysis!X$4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="49"/>
-      <c r="M6" s="49"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
@@ -3336,15 +3336,15 @@
         <f>Analysis!O3</f>
         <v/>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49"/>
-      <c r="M7" s="49"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
@@ -3354,15 +3354,15 @@
         <f>Analysis!P3</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E8" s="49"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="49"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="49"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="49"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="49"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="33" t="s">
@@ -4500,13 +4500,13 @@
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
       <c r="F17" s="42"/>
-      <c r="G17" s="52" t="s">
+      <c r="G17" s="45" t="s">
         <v>133</v>
       </c>
-      <c r="H17" s="51"/>
-      <c r="I17" s="51"/>
-      <c r="J17" s="51"/>
-      <c r="K17" s="51"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="46"/>
+      <c r="K17" s="46"/>
       <c r="L17" s="42"/>
       <c r="M17" s="42"/>
       <c r="N17" s="42"/>
@@ -4523,21 +4523,21 @@
       <c r="Y17" s="42"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="G18" s="51"/>
-      <c r="H18" s="51"/>
-      <c r="I18" s="51"/>
-      <c r="J18" s="51"/>
-      <c r="K18" s="51"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="46"/>
+      <c r="K18" s="46"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>52</v>
       </c>
-      <c r="G19" s="51"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="51"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="51"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -4549,11 +4549,11 @@
       <c r="C20" t="s">
         <v>55</v>
       </c>
-      <c r="G20" s="51"/>
-      <c r="H20" s="51"/>
-      <c r="I20" s="51"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="51"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="46"/>
+      <c r="K20" s="46"/>
     </row>
     <row r="21" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A21">
@@ -6692,10 +6692,10 @@
         <f>MAX(MAX(J14:J19)-MIN(J14:J19),MAX(K14:K19)-MIN(K14:K19))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O12" s="47" t="s">
+      <c r="O12" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="P12" s="47"/>
+      <c r="P12" s="51"/>
       <c r="Q12" s="13" t="s">
         <v>79</v>
       </c>
@@ -6851,11 +6851,11 @@
         <v/>
       </c>
       <c r="H15" s="1" t="e">
-        <f t="shared" ref="H15:H16" si="7">F$14-F15</f>
+        <f>F15-F$14</f>
         <v>#VALUE!</v>
       </c>
       <c r="I15" s="1" t="e">
-        <f t="shared" ref="I15:I16" si="8">G$14-G15</f>
+        <f>G15-G$14</f>
         <v>#VALUE!</v>
       </c>
       <c r="J15" s="1" t="e">
@@ -6867,11 +6867,11 @@
         <v>#VALUE!</v>
       </c>
       <c r="L15" s="5">
-        <f t="shared" ref="L15:L16" si="9">L$14*COS(C15*PI()/180)+M$14*SIN(C15*PI()/180)</f>
+        <f t="shared" ref="L15:L16" si="7">L$14*COS(C15*PI()/180)+M$14*SIN(C15*PI()/180)</f>
         <v>-1.0173001015936742</v>
       </c>
       <c r="M15" s="6">
-        <f t="shared" ref="M15:M16" si="10">M$14*COS(C15*PI()/180)-L$14*SIN(C15*PI()/180)</f>
+        <f t="shared" ref="M15:M16" si="8">M$14*COS(C15*PI()/180)-L$14*SIN(C15*PI()/180)</f>
         <v>-0.9823952887191082</v>
       </c>
       <c r="P15" s="7" t="e">
@@ -6883,7 +6883,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="R15" s="12" t="str">
-        <f t="shared" ref="R15:R20" si="11">IF(OR(D15="",E15=""),"",P15^2+Q15^2)</f>
+        <f t="shared" ref="R15:R20" si="9">IF(OR(D15="",E15=""),"",P15^2+Q15^2)</f>
         <v/>
       </c>
       <c r="U15" s="1"/>
@@ -6918,11 +6918,11 @@
         <v/>
       </c>
       <c r="H16" s="1" t="e">
-        <f t="shared" si="7"/>
+        <f>F16-F$14</f>
         <v>#VALUE!</v>
       </c>
       <c r="I16" s="1" t="e">
-        <f t="shared" si="8"/>
+        <f>G16-G$14</f>
         <v>#VALUE!</v>
       </c>
       <c r="J16" s="1" t="e">
@@ -6934,11 +6934,11 @@
         <v>#VALUE!</v>
       </c>
       <c r="L16" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>-1.0173001015936742</v>
       </c>
       <c r="M16" s="8">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>-0.9823952887191082</v>
       </c>
       <c r="P16" s="7" t="e">
@@ -6950,7 +6950,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="R16" s="12" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U16" s="1"/>
@@ -6969,7 +6969,7 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="8"/>
       <c r="R17" s="12" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U17" s="1"/>
@@ -6988,7 +6988,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="8"/>
       <c r="R18" s="12" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U18" s="1"/>
@@ -7007,7 +7007,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="8"/>
       <c r="R19" s="12" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U19" s="1"/>
@@ -7026,36 +7026,36 @@
       <c r="P20" s="9"/>
       <c r="Q20" s="10"/>
       <c r="R20" s="12" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U20" s="1"/>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="L21" s="43" t="s">
+      <c r="L21" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="M21" s="44"/>
-      <c r="P21" s="43" t="s">
+      <c r="M21" s="48"/>
+      <c r="P21" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="Q21" s="44"/>
-      <c r="R21" s="43" t="s">
+      <c r="Q21" s="48"/>
+      <c r="R21" s="47" t="s">
         <v>82</v>
       </c>
-      <c r="S21" s="44"/>
+      <c r="S21" s="48"/>
     </row>
     <row r="22" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>Data!A19</f>
         <v>ballCBCT</v>
       </c>
-      <c r="L22" s="45"/>
-      <c r="M22" s="46"/>
-      <c r="P22" s="45"/>
-      <c r="Q22" s="46"/>
-      <c r="R22" s="45"/>
-      <c r="S22" s="46"/>
+      <c r="L22" s="49"/>
+      <c r="M22" s="50"/>
+      <c r="P22" s="49"/>
+      <c r="Q22" s="50"/>
+      <c r="R22" s="49"/>
+      <c r="S22" s="50"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
@@ -7108,11 +7108,11 @@
         <v>0</v>
       </c>
       <c r="B27" s="1">
-        <f t="shared" ref="B27:C27" si="12">-B24</f>
+        <f t="shared" ref="B27:C27" si="10">-B24</f>
         <v>0</v>
       </c>
       <c r="C27" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -7145,12 +7145,12 @@
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H2" s="48" t="s">
+      <c r="H2" s="52" t="s">
         <v>117</v>
       </c>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
       <c r="L2" s="35">
         <f>MAX(L4:L6)</f>
         <v>0</v>

</xml_diff>